<commit_message>
feat(reponse-2): approfondissement - schemas, recalculs IR/PS, taux effectifs, fourchettes
- Schemas SVG (nouveau type de section 'schema' dans AnalyseContent): chronologie,
  arbre de dependance (tout depend de la reconstitution), roles des co-gerants
  (maitre unique), effet de levier x4, barres de taux effectif, waterfall du supplement
- Recalcul integral IR/PS annee par annee par associe (IR bareme + 40% + interets + PS),
  taux effectifs 73% (Behem) et 84% (Pasteur)
- Verification QPC: l'assiette sociale exclut bien le coefficient 1,25 (conforme) -
  correction honnete, pas de fausse faille
- Anticipation des contre-arguments du fisc (944/21302, conso>achats, maitre de l'affaire)
- Fourchettes de scenarios; Excel enrichis

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YXeuvw5FcfiJESGdc5g8m6
</commit_message>
<xml_diff>
--- a/public/documents/pieces-reponse-2/R2-chiffrage-behem.xlsx
+++ b/public/documents/pieces-reponse-2/R2-chiffrage-behem.xlsx
@@ -57,27 +57,13 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00DDDDDD"/>
-      </left>
-      <right style="thin">
-        <color rgb="00DDDDDD"/>
-      </right>
-      <top style="thin">
-        <color rgb="00DDDDDD"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00DDDDDD"/>
-      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -86,7 +72,7 @@
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -469,14 +455,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -499,17 +489,37 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Assiette IR (× 1,25)</t>
+          <t>Assiette IR (×1,25)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Supplément d'impôt notifié</t>
+          <t>IR au barème</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Part</t>
+          <t>Majoration 40 %</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Intérêts</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Prélèv. sociaux et ajust.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Supplément</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Taux effectif</t>
         </is>
       </c>
     </row>
@@ -526,10 +536,24 @@
         <v>120771</v>
       </c>
       <c r="D4" s="3" t="n">
+        <v>36215</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>14356</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>1974</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>21314</v>
+      </c>
+      <c r="H4" s="3" t="n">
         <v>73859</v>
       </c>
-      <c r="E4" s="4" t="n">
-        <v>42.8</v>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>76,4 %</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -544,11 +568,31 @@
       <c r="C5" s="3" t="n">
         <v>86790</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>n.c.</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>9820</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>n.c.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>n.c.</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="n">
         <v>48124</v>
       </c>
-      <c r="E5" s="4" t="n">
-        <v>27.9</v>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>69,3 %</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -564,10 +608,24 @@
         <v>87330</v>
       </c>
       <c r="D6" s="3" t="n">
+        <v>25336</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>9756</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>15433</v>
+      </c>
+      <c r="H6" s="3" t="n">
         <v>50720</v>
       </c>
-      <c r="E6" s="4" t="n">
-        <v>29.4</v>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>72,6 %</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -582,45 +640,62 @@
       <c r="C7" s="6" t="n">
         <v>294891</v>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="6" t="n">
+        <v>33932</v>
+      </c>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="n"/>
+      <c r="H7" s="6" t="n">
         <v>172703</v>
       </c>
-      <c r="E7" s="7" t="n"/>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>73,2 %</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Contrôle somme : 73859 + 48124 + 50720 = 172703 €</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>Chaque supplément cumule : impôt sur le revenu (barème, assiette distribuée × 1,25), CSG/CRDS, prélèvement de solidarité, majoration de 40 % (art. 1729) et intérêts de retard.</t>
+          <t>Contrôle : 73859 + 48124 + 50720 = 172703 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Nombre de parts : 1,00 / 1,00 / 1,00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>Base des prélèvements sociaux 2023 = 86 407 € (sans le coefficient 1,25) → conforme à la réserve du Conseil constitutionnel (2017-643/650 QPC).</t>
+          <t>Taux effectif = supplément / somme réputée distribuée (base RCM). Il atteint 73,2 % en moyenne.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>Montants repris des pages « CONSEQUENCES FINANCIERES » de la proposition personnelle BEHEM du 19/10/2026.</t>
+          <t>Base des prélèvements sociaux 2023 = 86 407 € (sans le coefficient 1,25) → conforme à la réserve QPC 2017-643/650.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>n.c. : composante non lue à l'OCR sur l'année 2024 ; le supplément total (48 124 €) et la base sont certains.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="A14:I14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>